<commit_message>
dont know whats happening
</commit_message>
<xml_diff>
--- a/rvfvmetadataandsequences.xlsx
+++ b/rvfvmetadataandsequences.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elleadams/Documents/GitHub/EPID8200Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7943FD76-3E4C-5A47-B1CC-48AE7213E7FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{54097ACB-F908-CE40-8F0F-D915E09ECAAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11980" yWindow="500" windowWidth="16440" windowHeight="16580" xr2:uid="{67DE6D1E-CCA3-094A-9646-E293AFF48C5C}"/>
+    <workbookView xWindow="11980" yWindow="520" windowWidth="16440" windowHeight="16580" xr2:uid="{67DE6D1E-CCA3-094A-9646-E293AFF48C5C}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -2960,7 +2960,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="mm/dd/yy;@"/>
+    <numFmt numFmtId="164" formatCode="mm/dd/yy;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -3000,10 +3000,10 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -18681,6 +18681,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ignoredErrors>
+    <ignoredError sqref="D480" twoDigitTextYear="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
i really changed one date to 2044 instead of 1944 ugh
</commit_message>
<xml_diff>
--- a/rvfvmetadataandsequences.xlsx
+++ b/rvfvmetadataandsequences.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elleadams/Documents/GitHub/EPID8200Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{82917EB3-7711-9641-BAD0-45153619FF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F419C3F-C273-F540-94BC-8099E8ED88A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11940" yWindow="540" windowWidth="16440" windowHeight="16580" xr2:uid="{67DE6D1E-CCA3-094A-9646-E293AFF48C5C}"/>
+    <workbookView xWindow="11940" yWindow="500" windowWidth="16440" windowHeight="16580" xr2:uid="{67DE6D1E-CCA3-094A-9646-E293AFF48C5C}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -3635,7 +3635,7 @@
         <v>934</v>
       </c>
       <c r="D13" s="3">
-        <v>52597</v>
+        <v>16072</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>934</v>

</xml_diff>